<commit_message>
Migracion de app local a app web
</commit_message>
<xml_diff>
--- a/resultados/facturas_lubrisol(1).xlsx
+++ b/resultados/facturas_lubrisol(1).xlsx
@@ -449,23 +449,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="35" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
   </cols>
@@ -555,112 +555,135 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>1389</t>
+          <t>1608</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>1389</t>
+          <t>1608</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>GMB ARQUINOX SAS</t>
+          <t>CNC MECANIZADOS OROS SAS</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>GMB ARQUINOX SAS</t>
+          <t>CNC MECANIZADOS OROS SAS</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>CL 2 73 B 39, Bogotá, 11001</t>
+          <t>TV 65 B NO. 1 - 57, Bogotá, 111621</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr"/>
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>900495221</t>
+          <t>901788378</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>usuario pos</t>
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>272600.01</v>
+        <v>95900.00999999999</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>LUBSYNT BLK 1 Gal. (2.0 x 114,537.82) = 272,600.01</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr"/>
-      <c r="O2" s="3" t="inlineStr"/>
+          <t>LUBGUIAS No. 2 1 Gal. (1.0 x 80,588.24) = 95,900.01</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>pvcarvajal@lubrisoldecolombia.com</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>522854991</t>
+        </is>
+      </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>80102010</t>
+          <t>80102009</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1388</t>
+          <t>1607</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1388</t>
+          <t>1607</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SIN NOMBRE</t>
+          <t>S Y G METALIZACION S.A.S.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SIN NOMBRE</t>
+          <t>S Y G METALIZACION S.A.S.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CL 24 SUR 69 C 32, Bogotá, 110841</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>222222222222</t>
+          <t>900192440</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>usuario pos</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>272600.01</v>
+        <v>136300.01</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>LUBSYNT BLK 1 Gal. (2.0 x 114,537.82) = 272,600.01</t>
+          <t>LUBSYNT BLK 1 Gal. (1.0 x 114,537.82) = 136,300.01</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>pvcarvajal@lubrisoldecolombia.com</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>522854991</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -672,605 +695,394 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1387</t>
+          <t>8780</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1387</t>
+          <t>8780</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>COLORHOME SAS</t>
+          <t>DANIELA STFANNY RINCON ORTIZ</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>COLORHOME SAS</t>
+          <t>DANIELA STFANNY RINCON ORTIZ</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>CR 70 22 90 SUR, Bogotá, 110831</t>
+          <t>CR 81 F # 68 - 34 sur, Bogotá, 110741</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>901649078</t>
+          <t>1012399389</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>ID: 660</t>
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>95900.00999999999</v>
+        <v>444500</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0</v>
+        <v>444500</v>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>LUBGUIAS No. 2 1 Gal. (1.0 x 80,588.24) = 95,900.01</t>
+          <t>LUBTHERM 27 Aceite térmico 1/5 Gal (19 litros) (1.0 x 373,529.41) = 444,500.0</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>80102009</t>
+          <t>50101164</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1386</t>
+          <t>8779</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1386</t>
+          <t>8779</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>BINGEM SAS</t>
+          <t>ROYTEC SAS</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BINGEM SAS</t>
+          <t>ROYTEC SAS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CL 56A 74 08, Bogotá, 111021</t>
+          <t>CR 68 A 3 28 SUR, Bogotá, 111631</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>901298415</t>
+          <t>901152522</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>ID: 660</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>103400</v>
+        <v>434830.46</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>434830.46</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>LUBGEAR GX SAE 90 1 Gal. (1.0 x 86,890.76) = 103,400.0</t>
+          <t>LUB HD 46 Aceite hidráulico antidesgaste 1/5 Gal (19 litros) (1.0 x 374,369.75) = 445,500.0</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>80102023</t>
+          <t>50101128</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>1385</t>
+          <t>8778</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>1385</t>
+          <t>8778</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>AT&amp;T SOLUCIONES METALMECANICAS SAS</t>
+          <t>COMPAÑIA COMUNITARIA METALMECANICA SAS</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>AT&amp;T SOLUCIONES METALMECANICAS SAS</t>
+          <t>COMPAÑIA COMUNITARIA METALMECANICA SAS</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>TV 65 A 1 A 33, Bogotá, 111611</t>
+          <t>CR 32 No 38A - 45 SUR, Bogotá, 00000</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>901137874</t>
+          <t>800066320</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>Andrés Gabino Porras Amaya</t>
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>136300.01</v>
+        <v>424300</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0</v>
+        <v>424300</v>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>LUBSYNT BLK 1 Gal. (1.0 x 114,537.82) = 136,300.01</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr"/>
-      <c r="O6" s="3" t="inlineStr"/>
+          <t>LUB HD 46 Aceite hidráulico antidesgaste 1/5 Gal (19 litros) (1.0 x 356,554.62) = 424,300.0</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>andresgabinopor@gmail.com</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>1015460667</t>
+        </is>
+      </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>80102010</t>
+          <t>50101128</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1384</t>
+          <t>8777</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1384</t>
+          <t>8777</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SIN NOMBRE</t>
+          <t>S Y G METALIZACION S.A.S.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SIN NOMBRE</t>
+          <t>S Y G METALIZACION S.A.S.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CL 24 SUR 69 C 32, Bogotá, 110841</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>222222222222</t>
+          <t>900192440</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>Andrés Gabino Porras Amaya</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>112800</v>
+        <v>637900</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>637900</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>EMULSOL 40 1 Gal. (1.0 x 94,789.92) = 112,800.0</t>
+          <t>LUBSYNT BLK Fluido sintético para mecanizado 1/5 Gal (19 litros) (1.0 x 536,050.42) = 637,900.0</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>andresgabinopor@gmail.com</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1015460667</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>80102002</t>
+          <t>50101119</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>1383</t>
+          <t>8776</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>1383</t>
+          <t>8776</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>CARIN LUVOV PARDO DIAZ</t>
+          <t>FTCAR S.A.S.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>CARIN LUVOV PARDO DIAZ</t>
+          <t>FTCAR S.A.S.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>CL 42 A SUR 99 F 22, Bogotá, 110881</t>
+          <t>CL 12 BIS # 71 G - 25 VILLA ALSACIA, Mosquera, 110831</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>1022395673</t>
+          <t>830136884</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>ID: 771</t>
+          <t>ID: 660</t>
         </is>
       </c>
       <c r="K8" s="3" t="n">
-        <v>136300.01</v>
+        <v>1075300.01</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0</v>
+        <v>1075300.01</v>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>LUBSYNT BLK 1 Gal. (1.0 x 114,537.82) = 136,300.01</t>
+          <t>LUBGUIAS 2 Aceite para guías y bancadas 1/5 Gal (19 litros) (1.0 x 367,563.03) = 437,400.01; LUBSYNT BLK Fluido sintético para mecanizado 1/5 Gal (19 litros) (1.0 x 536,050.42) = 637,900.0</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>80102010</t>
+          <t>50101159; 50101119</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8561</t>
+          <t>1606</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8561</t>
+          <t>1606</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MAQUINADOS Y MONTAJES S.A.S.</t>
+          <t>ARCRON BABY SAS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MAQUINADOS Y MONTAJES S.A.S.</t>
+          <t>ARCRON BABY SAS</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CR 16 No 60 - 14 BRR LA ESMERALDA, Girón, 00000</t>
+          <t>CR 70 31 79, Bogotá, 110841</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>800226501</t>
+          <t>900380065</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>ID: 660</t>
+          <t>usuario pos</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>637900</v>
+        <v>94200</v>
       </c>
       <c r="L9" t="n">
-        <v>637900</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>LUBSYNT BLK Fluido sintético para mecanizado 1/5 Gal (19 litros) (1.0 x 536,050.42) = 637,900.0</t>
+          <t>LUB HD 46 1 Gal. (1.0 x 79,159.66) = 94,200.0</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>pvcarvajal@lubrisoldecolombia.com</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>522854991</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>50101119</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>1382</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>1382</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>INDUSTRIAS RANDAL SAS</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>INDUSTRIAS RANDAL SAS</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>CL 35 SUR No. 70 B 12, Bogotá, 110841</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>830113529</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>ID: 771</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>71800.00999999999</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>LUBSYNT BLK 1/4 Galon (2.0 x 30,168.07) = 71,800.01</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr"/>
-      <c r="O10" s="3" t="inlineStr"/>
-      <c r="P10" s="3" t="inlineStr">
-        <is>
-          <t>80103010</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>8560</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>8560</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>AMANDA REINA QUIÑONEZ</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>AMANDA REINA QUIÑONEZ</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>CR 13 No. 23 - 76  BRR GIRARDOT, Bucaramanga, 00000</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>37816926</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>ID: 660</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>2407700</v>
-      </c>
-      <c r="L11" t="n">
-        <v>2407700</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>EMULSOL 40 Aceite soluble para mecanizado 1/5 Gal (19 litros) (3.0 x 424,117.65) = 1,514,100.01; SULFOMET C Aceite para corte y roscado 1/5 Gal (19 litros) (2.0 x 375,462.18) = 893,599.99</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>50101110; 50101091</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>8559</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>8559</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>PRODUCTOS Y PARTES SAS</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>PRODUCTOS Y PARTES SAS</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>CR 26 A No 26 - 79 SUR, Bogotá, 111511</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>900008238</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>ID: 666</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="n">
-        <v>1142600</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>1142600</v>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>LUBSYNT BLK Fluido sintético para mecanizado 1/5 Gal (19 litros) (1.0 x 536,050.42) = 637,900.0; EMULSOL 40 Aceite soluble para mecanizado 1/5 Gal (19 litros) (1.0 x 424,117.65) = 504,700.0</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr"/>
-      <c r="O12" s="3" t="inlineStr"/>
-      <c r="P12" s="3" t="inlineStr">
-        <is>
-          <t>50101119; 50101110</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>638</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>638</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ANGEL RAUL RINCON ROJAS</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>ANGEL RAUL RINCON ROJAS</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>CR 27 8 17 P1 BRR RICAURTE, Bogotá, 111411</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>80369062</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>ID: 771</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>35900</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>LUBSYNT BLK 1/4 Galon (1.0 x 30,168.07) = 35,900.0</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>80103010</t>
+          <t>80102005</t>
         </is>
       </c>
     </row>

</xml_diff>